<commit_message>
test: 建立统一开发 Fixture 并整合 Examples
- 新增 V1-24 Dev Fixture 基础资料库，为空白本地环境提供可重复使用的开发与验收数据
- 引入 10 张生成式测试图片，包括作品封面、人物头像与人物 Gallery 素材
- 建立 3 部虚构作品、2 位虚构人物及对应 Maker、Series、Genre、Tag、Asset 等关系数据
- 增加正常 Presentation Preference、默认回退和失效 Preference 等固定测试场景
- 为首选封面、首选头像、Asset 删除保护和失效引用提供可重复验收数据
- 新增 desktop:demo:seed、desktop:demo:reset 与 desktop:demo:clean 命令
- 将运行时 Fixture 隔离到 var/dev-fixture-library，避免测试操作修改 Git 中的模板数据
- 新增 validate:fixture，并纳入 pnpm check，校验 JSON 引用、Asset 文件、SHA-256、Presentation Preference 与测试场景完整性
- 将原 examples/works 与 examples/people 的旧单文件示例合并进统一 Dev Fixture
- 统一 imports、settings、shared-packs 与 dev-library 的虚构测试数据模型
- 将导入示例改为 LX 系列 Fixture 数据，使已有 Work 匹配与字段差异审核可以直接复现
- 增加 Private 与 Shared Pack 同 ID 不同值的优先级测试场景
- 更新 Examples、Fixture、AGENTS、README、MANIFEST、PROJECT_STATUS 与 CHANGELOG 文档
- 保持产品版本为 0.1.24，本次仅调整开发测试基础设施
- 验证通过 validate:fixture、pnpm check、desktop Rust check 与 Desktop 实机运行
</commit_message>
<xml_diff>
--- a/examples/imports/sample-works.xlsx
+++ b/examples/imports/sample-works.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="作品" sheetId="1" r:id="R62a585524c5f454a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="作品" sheetId="1" r:id="R1322901af33043fa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -39,7 +39,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="6">
+  <x:cellXfs count="7">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -50,6 +50,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -310,76 +311,78 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="5" t="str">
-        <x:v>DEMO-IMPORT-003</x:v>
+        <x:v>LX-408</x:v>
       </x:c>
       <x:c r="B2" s="5" t="str">
-        <x:v>星降る午後</x:v>
+        <x:v>晨光笔记</x:v>
       </x:c>
       <x:c r="C2" s="5" t="str">
-        <x:v>星降る午後</x:v>
+        <x:v>朝のノート</x:v>
       </x:c>
       <x:c r="D2" s="5" t="str">
-        <x:v>2026-08-21</x:v>
+        <x:v>2026-09-05</x:v>
       </x:c>
       <x:c r="E2" s="5" t="n">
         <x:v>118</x:v>
       </x:c>
       <x:c r="F2" s="5" t="str">
-        <x:v>星野みづき|白石りん</x:v>
+        <x:v>立花りな</x:v>
       </x:c>
       <x:c r="G2" s="5" t="str">
         <x:v>架空監督A</x:v>
       </x:c>
       <x:c r="H2" s="5" t="str">
-        <x:v>Aurora Works</x:v>
+        <x:v>ルーメン・フィクスチャー</x:v>
       </x:c>
       <x:c r="I2" s="5" t="str">
-        <x:v>Aurora Label</x:v>
+        <x:v>LX テストレーベル</x:v>
       </x:c>
       <x:c r="J2" s="5" t="str">
-        <x:v>夏の記憶</x:v>
+        <x:v>ビジュアル・ノーツ</x:v>
       </x:c>
       <x:c r="K2" s="5" t="str">
-        <x:v>ドラマ|制服</x:v>
+        <x:v>ドラマ|OL</x:v>
       </x:c>
       <x:c r="L2" s="5" t="str">
-        <x:v>待整理</x:v>
+        <x:v>要確認</x:v>
       </x:c>
       <x:c r="M2" s="5" t="str">
-        <x:v>co_starring</x:v>
+        <x:v>image_video</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="5" t="str">
-        <x:v>DEMO-IMPORT-004</x:v>
+        <x:v>LX-409</x:v>
       </x:c>
       <x:c r="B3" s="5" t="str">
-        <x:v>静かな海辺</x:v>
+        <x:v>两人的黄昏</x:v>
       </x:c>
       <x:c r="C3" s="5" t="str">
-        <x:v>静かな海辺</x:v>
+        <x:v>ふたりの夕暮れ</x:v>
       </x:c>
       <x:c r="D3" s="5" t="str">
-        <x:v>2026-08-28</x:v>
+        <x:v>2026-09-06</x:v>
       </x:c>
       <x:c r="E3" s="5" t="n">
         <x:v>96</x:v>
       </x:c>
       <x:c r="F3" s="5" t="str">
-        <x:v>白石りん</x:v>
+        <x:v>水野あいこ|立花りな</x:v>
       </x:c>
       <x:c r="G3" s="5" t="str">
         <x:v>架空監督B</x:v>
       </x:c>
       <x:c r="H3" s="5" t="str">
-        <x:v>North Studio</x:v>
+        <x:v>ルーメン・フィクスチャー</x:v>
       </x:c>
       <x:c r="I3" s="5" t="str">
-        <x:v>North Label</x:v>
-      </x:c>
-      <x:c r="J3" s="5" t="str"/>
+        <x:v>LX テストレーベル</x:v>
+      </x:c>
+      <x:c r="J3" s="5" t="str">
+        <x:v>ビジュアル・ノーツ</x:v>
+      </x:c>
       <x:c r="K3" s="5" t="str">
-        <x:v>イメージ|海辺</x:v>
+        <x:v>ドラマ|スレンダー</x:v>
       </x:c>
       <x:c r="L3" s="5" t="str">
         <x:v>お気に入り</x:v>

</xml_diff>